<commit_message>
updated api state transition rules
</commit_message>
<xml_diff>
--- a/states_reason.xlsx
+++ b/states_reason.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Inlogic_Projects\AI_Testing\ado_board_deva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44941F6-E17F-4127-94B3-3B23E59CDB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2FA5B2-9C7C-4725-8733-BB9D8F00D4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,9 +72,6 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>Ready for Release</t>
-  </si>
-  <si>
     <t>Code Review</t>
   </si>
   <si>
@@ -118,6 +115,9 @@
   </si>
   <si>
     <t>To Do</t>
+  </si>
+  <si>
+    <t>Ready to Release</t>
   </si>
 </sst>
 </file>
@@ -697,7 +697,7 @@
         <v>4</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -717,7 +717,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -734,7 +734,7 @@
         <v>8</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>9</v>
@@ -757,7 +757,7 @@
         <v>9</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -782,49 +782,49 @@
     </row>
     <row r="8" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="16" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="H8" s="17" t="s">
         <v>16</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>18</v>
-      </c>
       <c r="E9" s="22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="27"/>
     </row>
     <row r="10" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="20"/>
       <c r="C10" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="28"/>
     </row>
@@ -843,10 +843,10 @@
       <c r="B12" s="20"/>
       <c r="C12" s="14"/>
       <c r="D12" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" s="28"/>
     </row>
@@ -854,10 +854,10 @@
       <c r="B13" s="20"/>
       <c r="C13" s="14"/>
       <c r="D13" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F13" s="28"/>
     </row>
@@ -865,10 +865,10 @@
       <c r="B14" s="20"/>
       <c r="C14" s="14"/>
       <c r="D14" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F14" s="28"/>
     </row>
@@ -876,10 +876,10 @@
       <c r="B15" s="20"/>
       <c r="C15" s="14"/>
       <c r="D15" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F15" s="28"/>
     </row>
@@ -887,10 +887,10 @@
       <c r="B16" s="20"/>
       <c r="C16" s="14"/>
       <c r="D16" s="21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F16" s="28"/>
     </row>
@@ -898,10 +898,10 @@
       <c r="B17" s="20"/>
       <c r="C17" s="14"/>
       <c r="D17" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="25" t="s">
         <v>25</v>
-      </c>
-      <c r="E17" s="25" t="s">
-        <v>26</v>
       </c>
       <c r="F17" s="28"/>
     </row>
@@ -910,7 +910,7 @@
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F18" s="29"/>
     </row>

</xml_diff>

<commit_message>
update the user stories state transition rule new
</commit_message>
<xml_diff>
--- a/states_reason.xlsx
+++ b/states_reason.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Inlogic_Projects\AI_Testing\ado_board_deva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2FA5B2-9C7C-4725-8733-BB9D8F00D4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7003096-9076-4EC0-AD64-A5484A0780F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="31">
   <si>
     <t>EPIC</t>
   </si>
@@ -817,7 +817,7 @@
     </row>
     <row r="10" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="20"/>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="26" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -908,7 +908,9 @@
     <row r="18" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="20"/>
       <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
+      <c r="D18" s="26" t="s">
+        <v>16</v>
+      </c>
       <c r="E18" s="25" t="s">
         <v>24</v>
       </c>

</xml_diff>